<commit_message>
Add apres-ski addresses and Google Maps links
</commit_message>
<xml_diff>
--- a/data/apres_ski.xlsx
+++ b/data/apres_ski.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ethz-my.sharepoint.com/personal/vihrap_ethz_ch/Documents/MSc Semester 2/Intro to Python/Final Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chealenberry/Downloads/ETH Zürich/Spring Semester 2026/Intro to Python/winter-activities-switzerland/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{B6F5CBEA-F674-CB44-8D0F-73400C6EA4BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44F30BDD-EA0F-254B-90C5-5330C350A6DA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FAA2997-9C4C-4F43-8DF9-675E52FED66E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="940" windowWidth="14880" windowHeight="17200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="140" yWindow="500" windowWidth="14880" windowHeight="16480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
   <si>
     <t>Suggested Geocoding Query</t>
   </si>
@@ -272,14 +272,145 @@
   </si>
   <si>
     <t>name</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>Dorfstrasse 91, 6561 Ischgl, Austria</t>
+  </si>
+  <si>
+    <t>Dorfstrasse 74, 6561 Ischgl, Austria</t>
+  </si>
+  <si>
+    <t>Paznauner Taja 2, 6561 Ischgl, Austria</t>
+  </si>
+  <si>
+    <t>Kleine Scheidegg, 3823 Grindelwald, Switzerland</t>
+  </si>
+  <si>
+    <t>Tschuggenhütte, 7050 Arosa, Switzerland</t>
+  </si>
+  <si>
+    <t>Dieschen Seura 7, 7078 Lenzerheide, Switzerland</t>
+  </si>
+  <si>
+    <t>Stätz Damiez, 7075 Churwalden, Switzerland</t>
+  </si>
+  <si>
+    <t>Ritistrasse 156, 3997 Bellwald, Switzerland</t>
+  </si>
+  <si>
+    <t>Via Tinus 82, 7500 St. Moritz, Switzerland</t>
+  </si>
+  <si>
+    <t>Marguns, 7505 Celerina, Switzerland</t>
+  </si>
+  <si>
+    <t>Route du Téléphérique 32, 3963 Crans-Montana, Switzerland</t>
+  </si>
+  <si>
+    <t>Cry d'Er, 3963 Crans-Montana, Switzerland</t>
+  </si>
+  <si>
+    <t>Gerschnistrasse 12, 6390 Engelberg, Switzerland</t>
+  </si>
+  <si>
+    <t>Trübsee, 6390 Engelberg, Switzerland</t>
+  </si>
+  <si>
+    <t>Aroleidwald, 3920 Zermatt, Switzerland</t>
+  </si>
+  <si>
+    <t>Riedweg 156, 3920 Zermatt, Switzerland</t>
+  </si>
+  <si>
+    <t>Skistrasse 26, 7270 Davos, Switzerland</t>
+  </si>
+  <si>
+    <t>Skistrasse 9A, 7270 Davos Platz, Switzerland</t>
+  </si>
+  <si>
+    <t>Via Murschetg 15, 7032 Laax, Switzerland</t>
+  </si>
+  <si>
+    <t>Talstation Flims, 7017 Flims, Switzerland</t>
+  </si>
+  <si>
+    <t>Rütistrasse 9, 6490 Andermatt, Switzerland</t>
+  </si>
+  <si>
+    <t>Oberalpstrasse 28, 6490 Andermatt, Switzerland</t>
+  </si>
+  <si>
+    <t>Pale Soura 2, 7460 Savognin, Switzerland</t>
+  </si>
+  <si>
+    <t>7460 Savognin, Switzerland</t>
+  </si>
+  <si>
+    <t>Gletscherstrasse 14, 3906 Saas-Fee, Switzerland</t>
+  </si>
+  <si>
+    <t>Dorfstrasse 43, 3906 Saas-Fee, Switzerland</t>
+  </si>
+  <si>
+    <t>Bahnhofstrasse 2, 7260 Davos Dorf, Switzerland</t>
+  </si>
+  <si>
+    <t>Totalp, 7260 Davos, Switzerland</t>
+  </si>
+  <si>
+    <t>Route du Golf, 1936 Verbier, Switzerland</t>
+  </si>
+  <si>
+    <t>3775 Lenk im Simmental, Switzerland</t>
+  </si>
+  <si>
+    <t>Fiescheralp 2, 3984 Fiesch, Switzerland</t>
+  </si>
+  <si>
+    <t>Via da Ftan 495, 7550 Scuol, Switzerland</t>
+  </si>
+  <si>
+    <t>Vordere Schwendistrasse 16, 9658 Wildhaus, Switzerland</t>
+  </si>
+  <si>
+    <t>Pizolstrasse 112, 7323 Wangs, Switzerland</t>
+  </si>
+  <si>
+    <t>Hohsaas Mountain Station, 3910 Saas-Grund, Switzerland</t>
+  </si>
+  <si>
+    <t>Flumserbergstrasse 151, 8897 Flums, Switzerland</t>
+  </si>
+  <si>
+    <t>Obmoos, 8767 Glarus Süd, Switzerland</t>
+  </si>
+  <si>
+    <t>Obere Gletscherstrasse 133, 3818 Grindelwald, Switzerland</t>
+  </si>
+  <si>
+    <t>Madrisa-Hof, 7250 Klosters, Switzerland</t>
+  </si>
+  <si>
+    <t>1884 Villars-sur-Ollon, Switzerland</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -307,8 +438,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -611,14 +743,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="47.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>83</v>
       </c>
@@ -631,8 +764,11 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -645,8 +781,13 @@
       <c r="D2">
         <v>10.286929900000001</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -659,8 +800,11 @@
       <c r="D3">
         <v>10.2889748</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -673,8 +817,11 @@
       <c r="D4">
         <v>10.299228899999999</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -687,8 +834,11 @@
       <c r="D5">
         <v>7.9617680000000002</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -701,8 +851,11 @@
       <c r="D6">
         <v>9.6626288000000002</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -715,8 +868,11 @@
       <c r="D7">
         <v>9.5629372000000004</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -729,8 +885,11 @@
       <c r="D8">
         <v>9.5393264999999996</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -743,8 +902,11 @@
       <c r="D9">
         <v>8.1609280000000002</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -757,8 +919,11 @@
       <c r="D10">
         <v>9.8192587000000007</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -771,8 +936,11 @@
       <c r="D11">
         <v>9.8595229999999994</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E11" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -785,8 +953,11 @@
       <c r="D12">
         <v>7.4669132999999999</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E12" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -799,8 +970,11 @@
       <c r="D13">
         <v>7.4783727999999998</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -813,8 +987,11 @@
       <c r="D14">
         <v>8.3965233000000001</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E14" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -827,8 +1004,11 @@
       <c r="D15">
         <v>8.0687859999999993</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -841,8 +1021,11 @@
       <c r="D16">
         <v>7.7374568000000004</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E16" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -855,8 +1038,11 @@
       <c r="D17">
         <v>7.7543012999999998</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E17" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -869,8 +1055,11 @@
       <c r="D18">
         <v>9.8229737000000004</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E18" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -883,8 +1072,11 @@
       <c r="D19">
         <v>9.8516750999999996</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E19" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -897,8 +1089,11 @@
       <c r="D20">
         <v>9.2637996999999999</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E20" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -911,8 +1106,11 @@
       <c r="D21">
         <v>9.2845800000000001</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E21" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -925,8 +1123,11 @@
       <c r="D22">
         <v>8.5938800000000004</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E22" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>45</v>
       </c>
@@ -939,8 +1140,11 @@
       <c r="D23">
         <v>8.6057281999999997</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E23" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>47</v>
       </c>
@@ -953,8 +1157,11 @@
       <c r="D24">
         <v>9.5982500000000002</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E24" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>49</v>
       </c>
@@ -967,8 +1174,11 @@
       <c r="D25">
         <v>9.5855937999999998</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>51</v>
       </c>
@@ -981,8 +1191,11 @@
       <c r="D26">
         <v>7.9261904999999997</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E26" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -995,8 +1208,11 @@
       <c r="D27">
         <v>7.9249444999999996</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E27" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>55</v>
       </c>
@@ -1009,8 +1225,11 @@
       <c r="D28">
         <v>9.8409528999999996</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E28" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>57</v>
       </c>
@@ -1023,8 +1242,11 @@
       <c r="D29">
         <v>9.8088574000000008</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E29" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>59</v>
       </c>
@@ -1037,8 +1259,11 @@
       <c r="D30">
         <v>7.2264062999999998</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E30" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>61</v>
       </c>
@@ -1051,8 +1276,11 @@
       <c r="D31">
         <v>7.4429800000000004</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E31" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>63</v>
       </c>
@@ -1065,8 +1293,11 @@
       <c r="D32">
         <v>8.1311</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -1079,8 +1310,11 @@
       <c r="D33">
         <v>10.2886218</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E33" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>67</v>
       </c>
@@ -1093,8 +1327,11 @@
       <c r="D34">
         <v>9.3548799999999996</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E34" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>69</v>
       </c>
@@ -1107,8 +1344,11 @@
       <c r="D35">
         <v>9.4340600000000006</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E35" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>71</v>
       </c>
@@ -1121,8 +1361,11 @@
       <c r="D36">
         <v>7.9910825000000001</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E36" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>73</v>
       </c>
@@ -1135,8 +1378,11 @@
       <c r="D37">
         <v>9.3034330000000001</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E37" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>75</v>
       </c>
@@ -1149,8 +1395,11 @@
       <c r="D38">
         <v>9.1621892999999996</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E38" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>77</v>
       </c>
@@ -1163,8 +1412,11 @@
       <c r="D39">
         <v>8.0627148000000002</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E39" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>79</v>
       </c>
@@ -1177,8 +1429,11 @@
       <c r="D40">
         <v>9.8815100000000005</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E40" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>81</v>
       </c>
@@ -1190,6 +1445,9 @@
       </c>
       <c r="D41">
         <v>7.2162100000000002</v>
+      </c>
+      <c r="E41" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>